<commit_message>
Add API analysis and audited test suites
</commit_message>
<xml_diff>
--- a/test-cases/login_test_cases_audited.xlsx
+++ b/test-cases/login_test_cases_audited.xlsx
@@ -10,7 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="login_cases" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metadata" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'login_cases'!$A$1:$X$46</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.001"/>
 </workbook>
 </file>
@@ -133,7 +135,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -167,6 +169,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -421,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:U41"/>
+  <dimension ref="A1:X46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="5" min="1" max="1"/>
@@ -444,6 +452,9 @@
     <col width="24" customWidth="1" style="5" min="19" max="19"/>
     <col width="48" customWidth="1" style="5" min="20" max="20"/>
     <col width="62" customWidth="1" style="6" min="21" max="21"/>
+    <col width="58" customWidth="1" style="6" min="22" max="22"/>
+    <col width="58" customWidth="1" style="6" min="23" max="23"/>
+    <col width="58" customWidth="1" style="6" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.75" customHeight="1" s="6">
@@ -552,6 +563,21 @@
           <t>human_correction</t>
         </is>
       </c>
+      <c r="V1" s="7" t="inlineStr">
+        <is>
+          <t>extension_reason</t>
+        </is>
+      </c>
+      <c r="W1" s="7" t="inlineStr">
+        <is>
+          <t>ai_generated_gap</t>
+        </is>
+      </c>
+      <c r="X1" s="7" t="inlineStr">
+        <is>
+          <t>ai_miss_reason</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="41.25" customHeight="1" s="6">
       <c r="A2" s="9" t="inlineStr">
@@ -4393,7 +4419,598 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="12" t="inlineStr">
+        <is>
+          <t>LOGIN-EXT-001</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>POST /api/login</t>
+        </is>
+      </c>
+      <c r="C42" s="12" t="inlineStr">
+        <is>
+          <t>MANUAL_EXTENSION</t>
+        </is>
+      </c>
+      <c r="D42" s="12" t="inlineStr">
+        <is>
+          <t>FR-02</t>
+        </is>
+      </c>
+      <c r="E42" s="12" t="inlineStr">
+        <is>
+          <t>Token usability, Cross-request dependency</t>
+        </is>
+      </c>
+      <c r="F42" s="12" t="inlineStr">
+        <is>
+          <t>docs/api_specification.md - Authentication 1.2 POST /api/login; Users 2.1 GET /api/users/me requires Authorization: Bearer &lt;token&gt;</t>
+        </is>
+      </c>
+      <c r="G42" s="12" t="inlineStr">
+        <is>
+          <t>Kiểm tra token nhận từ login có thể được dùng cho API cần authentication.</t>
+        </is>
+      </c>
+      <c r="H42" s="12" t="inlineStr">
+        <is>
+          <t>Cần user hợp lệ tồn tại. Step 1 login bằng {{validUserEmail}}/{{validUserPassword}}. Step 2 dùng token response làm {{loginToken}} để gọi GET /api/users/me.</t>
+        </is>
+      </c>
+      <c r="I42" s="12" t="inlineStr">
+        <is>
+          <t>POST then GET</t>
+        </is>
+      </c>
+      <c r="J42" s="12" t="inlineStr">
+        <is>
+          <t>{{baseUrl}}/api/login then {{baseUrl}}/api/users/me</t>
+        </is>
+      </c>
+      <c r="K42" s="12" t="inlineStr">
+        <is>
+          <t>{"Content-Type":"application/json","X-Student-Id":"{{studentId}}"}; follow-up: {"Authorization":"Bearer {{loginToken}}","X-Student-Id":"{{studentId}}"}</t>
+        </is>
+      </c>
+      <c r="L42" s="12" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="M42" s="12" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="N42" s="12" t="inlineStr">
+        <is>
+          <t>Step 1 body: {"email":"{{validUserEmail}}","password":"{{validUserPassword}}"}; Step 2 body: none</t>
+        </is>
+      </c>
+      <c r="O42" s="12" t="inlineStr">
+        <is>
+          <t>login: 200; follow-up: SPEC_UNDEFINED</t>
+        </is>
+      </c>
+      <c r="P42" s="12" t="inlineStr">
+        <is>
+          <t>Login response phải có token string non-empty; token đó phải được API cần Authorization chấp nhận. Không ghi pass/fail nếu chưa execution.</t>
+        </is>
+      </c>
+      <c r="Q42" s="12" t="inlineStr">
+        <is>
+          <t>manual-extension,cross-request,security,schema</t>
+        </is>
+      </c>
+      <c r="R42" s="12" t="inlineStr">
+        <is>
+          <t>Spec login định nghĩa token nhưng GET /api/users/me không nêu success status cụ thể; follow-up status để SPEC_UNDEFINED.</t>
+        </is>
+      </c>
+      <c r="S42" s="12" t="inlineStr">
+        <is>
+          <t>STUDENT_DESIGNED</t>
+        </is>
+      </c>
+      <c r="T42" s="12" t="inlineStr">
+        <is>
+          <t>Manual extension do sinh viên chọn từ reports/analysis/login_extension_gaps.md; chưa execute, chưa pass/fail, chưa bug classification.</t>
+        </is>
+      </c>
+      <c r="U42" s="10" t="inlineStr"/>
+      <c r="V42" s="13" t="inlineStr">
+        <is>
+          <t>Gap 1 được chọn: cross-request token usability.</t>
+        </is>
+      </c>
+      <c r="W42" s="13" t="inlineStr">
+        <is>
+          <t>AI suite chỉ kiểm tra token tồn tại trong response, chưa kiểm tra token có usable cho API yêu cầu Authorization.</t>
+        </is>
+      </c>
+      <c r="X42" s="13" t="inlineStr">
+        <is>
+          <t>AI generation ban đầu tập trung vào single endpoint POST /api/login nên bỏ sót cross-request verification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t>LOGIN-EXT-002</t>
+        </is>
+      </c>
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>POST /api/login</t>
+        </is>
+      </c>
+      <c r="C43" s="12" t="inlineStr">
+        <is>
+          <t>MANUAL_EXTENSION</t>
+        </is>
+      </c>
+      <c r="D43" s="12" t="inlineStr">
+        <is>
+          <t>FR-02</t>
+        </is>
+      </c>
+      <c r="E43" s="12" t="inlineStr">
+        <is>
+          <t>Token/user consistency, Cross-user behavior, Information leakage</t>
+        </is>
+      </c>
+      <c r="F43" s="12" t="inlineStr">
+        <is>
+          <t>docs/api_specification.md - Authentication 1.2 POST /api/login; Users 2.1 GET /api/users/me</t>
+        </is>
+      </c>
+      <c r="G43" s="12" t="inlineStr">
+        <is>
+          <t>Kiểm tra thông tin user trong login response nhất quán với identity khi dùng token gọi GET /api/users/me.</t>
+        </is>
+      </c>
+      <c r="H43" s="12" t="inlineStr">
+        <is>
+          <t>Cần user hợp lệ tồn tại. Login lấy token và user object; sau đó gọi GET /api/users/me bằng token vừa nhận.</t>
+        </is>
+      </c>
+      <c r="I43" s="12" t="inlineStr">
+        <is>
+          <t>POST then GET</t>
+        </is>
+      </c>
+      <c r="J43" s="12" t="inlineStr">
+        <is>
+          <t>{{baseUrl}}/api/login then {{baseUrl}}/api/users/me</t>
+        </is>
+      </c>
+      <c r="K43" s="12" t="inlineStr">
+        <is>
+          <t>{"Content-Type":"application/json","X-Student-Id":"{{studentId}}"}; follow-up: {"Authorization":"Bearer {{loginToken}}","X-Student-Id":"{{studentId}}"}</t>
+        </is>
+      </c>
+      <c r="L43" s="12" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="M43" s="12" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="N43" s="12" t="inlineStr">
+        <is>
+          <t>Step 1 body: {"email":"{{validUserEmail}}","password":"{{validUserPassword}}"}; Step 2 body: none</t>
+        </is>
+      </c>
+      <c r="O43" s="12" t="inlineStr">
+        <is>
+          <t>login: 200; follow-up: SPEC_UNDEFINED</t>
+        </is>
+      </c>
+      <c r="P43" s="12" t="inlineStr">
+        <is>
+          <t>Nếu cả login user và /users/me response có cùng field định danh như id hoặc email, các giá trị đó phải nhất quán; không được trả user của tài khoản khác hoặc secret fields.</t>
+        </is>
+      </c>
+      <c r="Q43" s="12" t="inlineStr">
+        <is>
+          <t>manual-extension,cross-request,security,consistency</t>
+        </is>
+      </c>
+      <c r="R43" s="12" t="inlineStr">
+        <is>
+          <t>Spec chưa liệt kê field con của user và JWT claims, nên consistency chỉ assert trên các field thực tế cùng tồn tại trong response.</t>
+        </is>
+      </c>
+      <c r="S43" s="12" t="inlineStr">
+        <is>
+          <t>STUDENT_DESIGNED</t>
+        </is>
+      </c>
+      <c r="T43" s="12" t="inlineStr">
+        <is>
+          <t>Manual extension do sinh viên chọn từ reports/analysis/login_extension_gaps.md; chưa execute, chưa pass/fail, chưa bug classification.</t>
+        </is>
+      </c>
+      <c r="U43" s="10" t="inlineStr"/>
+      <c r="V43" s="13" t="inlineStr">
+        <is>
+          <t>Gap 2 được chọn: token/user consistency.</t>
+        </is>
+      </c>
+      <c r="W43" s="13" t="inlineStr">
+        <is>
+          <t>AI suite có schema check cho token và user riêng lẻ nhưng chưa đối chiếu identity giữa token và user.</t>
+        </is>
+      </c>
+      <c r="X43" s="13" t="inlineStr">
+        <is>
+          <t>AI có xu hướng tránh claim về JWT/user shape vì spec không mô tả chi tiết, nên bỏ sót consistency check gián tiếp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="12" t="inlineStr">
+        <is>
+          <t>LOGIN-EXT-003</t>
+        </is>
+      </c>
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>POST /api/login</t>
+        </is>
+      </c>
+      <c r="C44" s="12" t="inlineStr">
+        <is>
+          <t>MANUAL_EXTENSION</t>
+        </is>
+      </c>
+      <c r="D44" s="12" t="inlineStr">
+        <is>
+          <t>FR-02</t>
+        </is>
+      </c>
+      <c r="E44" s="12" t="inlineStr">
+        <is>
+          <t>Type confusion, Parser ambiguity, Injection</t>
+        </is>
+      </c>
+      <c r="F44" s="12" t="inlineStr">
+        <is>
+          <t>docs/api_specification.md - Authentication 1.2 request body email/password</t>
+        </is>
+      </c>
+      <c r="G44" s="12" t="inlineStr">
+        <is>
+          <t>Kiểm tra raw JSON có duplicate keys không gây bypass authentication hoặc parser ambiguity nguy hiểm.</t>
+        </is>
+      </c>
+      <c r="H44" s="12" t="inlineStr">
+        <is>
+          <t>Cần gửi raw JSON body trong Postman/Newman. Cần {{validUserEmail}}, {{validUserPassword}}, {{unknownEmail}}, và {{wrongPassword}}.</t>
+        </is>
+      </c>
+      <c r="I44" s="12" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="J44" s="12" t="inlineStr">
+        <is>
+          <t>{{baseUrl}}/api/login</t>
+        </is>
+      </c>
+      <c r="K44" s="12" t="inlineStr">
+        <is>
+          <t>{"Content-Type":"application/json","X-Student-Id":"{{studentId}}"}</t>
+        </is>
+      </c>
+      <c r="L44" s="12" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="M44" s="12" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="N44" s="12" t="inlineStr">
+        <is>
+          <t>{"email":"{{unknownEmail}}","email":"{{validUserEmail}}","password":"{{wrongPassword}}","password":"{{validUserPassword}}"}</t>
+        </is>
+      </c>
+      <c r="O44" s="12" t="inlineStr">
+        <is>
+          <t>SPEC_UNDEFINED</t>
+        </is>
+      </c>
+      <c r="P44" s="12" t="inlineStr">
+        <is>
+          <t>Ghi nhận parser dùng first key hay last key; request không được bypass auth ngoài cặp email/password hợp lệ mà parser thực sự sử dụng; response không lộ stack trace/internal error.</t>
+        </is>
+      </c>
+      <c r="Q44" s="12" t="inlineStr">
+        <is>
+          <t>manual-extension,security,parser,duplicate-keys,exploratory</t>
+        </is>
+      </c>
+      <c r="R44" s="12" t="inlineStr">
+        <is>
+          <t>JSON duplicate key behavior phụ thuộc parser/runtime và không được spec định nghĩa.</t>
+        </is>
+      </c>
+      <c r="S44" s="12" t="inlineStr">
+        <is>
+          <t>STUDENT_DESIGNED</t>
+        </is>
+      </c>
+      <c r="T44" s="12" t="inlineStr">
+        <is>
+          <t>Manual extension do sinh viên chọn từ reports/analysis/login_extension_gaps.md; chưa execute, chưa pass/fail, chưa bug classification.</t>
+        </is>
+      </c>
+      <c r="U44" s="10" t="inlineStr"/>
+      <c r="V44" s="13" t="inlineStr">
+        <is>
+          <t>Gap 3 được chọn: duplicate JSON keys.</t>
+        </is>
+      </c>
+      <c r="W44" s="13" t="inlineStr">
+        <is>
+          <t>AI suite có wrong type/object và malformed JSON nhưng chưa có raw JSON duplicate key case.</t>
+        </is>
+      </c>
+      <c r="X44" s="13" t="inlineStr">
+        <is>
+          <t>Duplicate key là edge case parser-level, thường bị bỏ sót khi AI sinh partition theo field riêng lẻ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t>LOGIN-EXT-004</t>
+        </is>
+      </c>
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>POST /api/login</t>
+        </is>
+      </c>
+      <c r="C45" s="12" t="inlineStr">
+        <is>
+          <t>MANUAL_EXTENSION</t>
+        </is>
+      </c>
+      <c r="D45" s="12" t="inlineStr">
+        <is>
+          <t>FR-02</t>
+        </is>
+      </c>
+      <c r="E45" s="12" t="inlineStr">
+        <is>
+          <t>Account enumeration</t>
+        </is>
+      </c>
+      <c r="F45" s="12" t="inlineStr">
+        <is>
+          <t>docs/api_specification.md - Authentication 1.2 POST /api/login; assignment FR-02 Login and account lockout</t>
+        </is>
+      </c>
+      <c r="G45" s="12" t="inlineStr">
+        <is>
+          <t>So sánh paired observation giữa unknown email và wrong password để đánh giá rủi ro account enumeration.</t>
+        </is>
+      </c>
+      <c r="H45" s="12" t="inlineStr">
+        <is>
+          <t>Cần {{validUserEmail}} tồn tại, {{wrongPassword}} sai với user đó, và {{unknownEmail}} không tồn tại. Chạy hai request liên tiếp trong cùng môi trường.</t>
+        </is>
+      </c>
+      <c r="I45" s="12" t="inlineStr">
+        <is>
+          <t>POST then POST</t>
+        </is>
+      </c>
+      <c r="J45" s="12" t="inlineStr">
+        <is>
+          <t>{{baseUrl}}/api/login then {{baseUrl}}/api/login</t>
+        </is>
+      </c>
+      <c r="K45" s="12" t="inlineStr">
+        <is>
+          <t>{"Content-Type":"application/json","X-Student-Id":"{{studentId}}"}</t>
+        </is>
+      </c>
+      <c r="L45" s="12" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="M45" s="12" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="N45" s="12" t="inlineStr">
+        <is>
+          <t>Request A: {"email":"{{unknownEmail}}","password":"{{wrongPassword}}"}; Request B: {"email":"{{validUserEmail}}","password":"{{wrongPassword}}"}</t>
+        </is>
+      </c>
+      <c r="O45" s="12" t="inlineStr">
+        <is>
+          <t>SPEC_UNDEFINED</t>
+        </is>
+      </c>
+      <c r="P45" s="12" t="inlineStr">
+        <is>
+          <t>Cả hai request không được trả token. Ghi nhận và so sánh status/message/response length/timing; nếu khác biệt thì đánh dấu observation để human analysis, không tự kết luận bug.</t>
+        </is>
+      </c>
+      <c r="Q45" s="12" t="inlineStr">
+        <is>
+          <t>manual-extension,security,account-enumeration,paired-observation</t>
+        </is>
+      </c>
+      <c r="R45" s="12" t="inlineStr">
+        <is>
+          <t>Spec không yêu cầu status/message giống nhau cho unknown email và wrong password.</t>
+        </is>
+      </c>
+      <c r="S45" s="12" t="inlineStr">
+        <is>
+          <t>STUDENT_DESIGNED</t>
+        </is>
+      </c>
+      <c r="T45" s="12" t="inlineStr">
+        <is>
+          <t>Manual extension do sinh viên chọn từ reports/analysis/login_extension_gaps.md; chưa execute, chưa pass/fail, chưa bug classification.</t>
+        </is>
+      </c>
+      <c r="U45" s="10" t="inlineStr"/>
+      <c r="V45" s="13" t="inlineStr">
+        <is>
+          <t>Gap 4 được chọn: paired account enumeration observation.</t>
+        </is>
+      </c>
+      <c r="W45" s="13" t="inlineStr">
+        <is>
+          <t>AI suite có các negative case riêng lẻ cho unknown email và wrong password nhưng chưa có paired comparison trong một flow.</t>
+        </is>
+      </c>
+      <c r="X45" s="13" t="inlineStr">
+        <is>
+          <t>AI sinh case theo từng input partition nên chưa gom thành observation có ý nghĩa security.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="12" t="inlineStr">
+        <is>
+          <t>LOGIN-EXT-005</t>
+        </is>
+      </c>
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>POST /api/login</t>
+        </is>
+      </c>
+      <c r="C46" s="12" t="inlineStr">
+        <is>
+          <t>MANUAL_EXTENSION</t>
+        </is>
+      </c>
+      <c r="D46" s="12" t="inlineStr">
+        <is>
+          <t>FR-02</t>
+        </is>
+      </c>
+      <c r="E46" s="12" t="inlineStr">
+        <is>
+          <t>Information leakage, HTTP parser error leakage</t>
+        </is>
+      </c>
+      <c r="F46" s="12" t="inlineStr">
+        <is>
+          <t>docs/api_specification.md - Authentication 1.2 POST /api/login; assignment security coverage</t>
+        </is>
+      </c>
+      <c r="G46" s="12" t="inlineStr">
+        <is>
+          <t>Kiểm tra malformed HTTP/JSON request không làm rò rỉ stack trace, framework error, file path, query, hoặc internal details.</t>
+        </is>
+      </c>
+      <c r="H46" s="12" t="inlineStr">
+        <is>
+          <t>Cần gửi raw malformed JSON hoặc body không parse được trong Postman/Newman.</t>
+        </is>
+      </c>
+      <c r="I46" s="12" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="J46" s="12" t="inlineStr">
+        <is>
+          <t>{{baseUrl}}/api/login</t>
+        </is>
+      </c>
+      <c r="K46" s="12" t="inlineStr">
+        <is>
+          <t>{"Content-Type":"application/json","X-Student-Id":"{{studentId}}"}</t>
+        </is>
+      </c>
+      <c r="L46" s="12" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="M46" s="12" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="N46" s="12" t="inlineStr">
+        <is>
+          <t>{"email":"{{validUserEmail}}","password":</t>
+        </is>
+      </c>
+      <c r="O46" s="12" t="inlineStr">
+        <is>
+          <t>SPEC_UNDEFINED</t>
+        </is>
+      </c>
+      <c r="P46" s="12" t="inlineStr">
+        <is>
+          <t>Response không được có token và không được lộ stack trace, file path, SQL query, framework exception, environment variable, hoặc internal implementation detail.</t>
+        </is>
+      </c>
+      <c r="Q46" s="12" t="inlineStr">
+        <is>
+          <t>manual-extension,security,http-parser,information-leakage</t>
+        </is>
+      </c>
+      <c r="R46" s="12" t="inlineStr">
+        <is>
+          <t>Spec không định nghĩa exact error status/schema cho malformed JSON.</t>
+        </is>
+      </c>
+      <c r="S46" s="12" t="inlineStr">
+        <is>
+          <t>STUDENT_DESIGNED</t>
+        </is>
+      </c>
+      <c r="T46" s="12" t="inlineStr">
+        <is>
+          <t>Manual extension do sinh viên chọn từ reports/analysis/login_extension_gaps.md; chưa execute, chưa pass/fail, chưa bug classification.</t>
+        </is>
+      </c>
+      <c r="U46" s="10" t="inlineStr"/>
+      <c r="V46" s="13" t="inlineStr">
+        <is>
+          <t>Gap 5 được chọn: HTTP parser error leakage.</t>
+        </is>
+      </c>
+      <c r="W46" s="13" t="inlineStr">
+        <is>
+          <t>AI suite có malformed JSON nhưng assertion chưa tập trung sâu vào các dạng internal leakage của parser/framework.</t>
+        </is>
+      </c>
+      <c r="X46" s="13" t="inlineStr">
+        <is>
+          <t>AI thường ghi assertion tổng quát "không crash" nên cần manual extension để làm rõ leakage signals cần kiểm tra.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:X46"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -4406,7 +5023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="28" customWidth="1" style="5" min="1" max="1"/>
@@ -4421,7 +5038,7 @@
       </c>
       <c r="B1" s="11" t="inlineStr">
         <is>
-          <t>PHASE_4_HUMAN_AUDIT</t>
+          <t>PHASE_5_HUMAN_EXTENSION</t>
         </is>
       </c>
     </row>
@@ -4516,6 +5133,42 @@
       <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Only rows with audit_status INVALID or INCOMPLETE; original AI content, audit_status, and audit_notes preserved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>manual_extension_count_login</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>manual_extension_ids_login</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>LOGIN-EXT-001..LOGIN-EXT-005</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>manual_extension_note</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Student-selected gaps appended as MANUAL_EXTENSION; no execution results recorded.</t>
         </is>
       </c>
     </row>

</xml_diff>